<commit_message>
Cleanup SQL backups and refactor reset/debug scripts for database workflow
</commit_message>
<xml_diff>
--- a/sql_scripts/which_tables_are_reference_tables.xlsx
+++ b/sql_scripts/which_tables_are_reference_tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dalia/Developer/RENERA/BADB_main/sql_scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5624E612-62E1-0C49-B653-425AF469BFAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA9280D-B6FC-0049-B07C-342FC2B9D9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="520" windowWidth="23360" windowHeight="14580" xr2:uid="{F3B5AF8C-65A7-724B-965E-90CE116FBB2D}"/>
   </bookViews>
@@ -167,10 +167,10 @@
     <t>clear</t>
   </si>
   <si>
-    <t>KEEP</t>
-  </si>
-  <si>
-    <t>KEEP for now</t>
+    <t>SEED DATA</t>
+  </si>
+  <si>
+    <t>REFERENCE</t>
   </si>
 </sst>
 </file>
@@ -646,7 +646,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
         <v>12</v>
@@ -662,7 +662,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
         <v>13</v>
@@ -686,7 +686,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -701,8 +701,8 @@
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>42</v>
+      <c r="A19" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="B19" t="s">
         <v>18</v>
@@ -718,31 +718,31 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B21" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>42</v>
+      <c r="A22" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="B22" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>42</v>
+      <c r="A23" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="B23" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>42</v>
+      <c r="A24" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="B24" t="s">
         <v>23</v>
@@ -774,7 +774,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
@@ -790,7 +790,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B30" t="s">
         <v>29</v>
@@ -798,7 +798,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B31" t="s">
         <v>30</v>
@@ -822,7 +822,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B34" t="s">
         <v>33</v>
@@ -830,7 +830,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B35" t="s">
         <v>34</v>
@@ -878,15 +878,15 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B41" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
-        <v>43</v>
+      <c r="A42" t="s">
+        <v>44</v>
       </c>
       <c r="B42" t="s">
         <v>41</v>

</xml_diff>